<commit_message>
mise a jour power bi
</commit_message>
<xml_diff>
--- a/dataset_bi/LogementsVacants_MEL_Exploitable.xlsx
+++ b/dataset_bi/LogementsVacants_MEL_Exploitable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Formation\crise_immo\Projet_crise_logement\dataset_bi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E35FAB11-2479-482B-952A-42CE3E4874C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F69C8D21-29D6-418D-B456-07C875C8C68B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -617,13 +617,14 @@
   <cols>
     <col min="1" max="1" width="14.109375" customWidth="1"/>
     <col min="2" max="2" width="32.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="21.21875" customWidth="1"/>
-    <col min="8" max="8" width="11.109375" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="20.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>